<commit_message>
Update reports 2026-09-03 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-03.xlsx
+++ b/gex_pivot_levels_2026-09-03.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Pivots'!$A$1:$H$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Pivots'!$A$1:$H$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -569,12 +569,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$8.49M</t>
+          <t>-$7.98M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$10.25M</t>
+          <t>+$9.63M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$2.63M</t>
+          <t>-$2.46M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$9.18M</t>
+          <t>+$8.60M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$10.85M</t>
+          <t>-$10.10M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$17.41M</t>
+          <t>+$16.21M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$11.25M</t>
+          <t>-$10.37M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$15.80M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$6.89M</t>
+          <t>-$6.49M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$19.05M</t>
+          <t>+$17.94M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>+$1.67M</t>
+          <t>+$1.69M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$27.76M</t>
+          <t>+$28.05M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>+$12.28M</t>
+          <t>+$12.41M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$19.23M</t>
+          <t>+$19.43M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -854,12 +854,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$662.78K</t>
+          <t>+$684.63K</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$9.09M</t>
+          <t>+$9.39M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -887,12 +887,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>+$10.25M</t>
+          <t>+$10.85M</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>+$17.04M</t>
+          <t>+$18.04M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -920,12 +920,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$3.67M</t>
+          <t>+$3.95M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$7.52M</t>
+          <t>+$8.10M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>+$16.55M</t>
+          <t>+$17.71M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$23.68M</t>
+          <t>+$25.35M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>+$6.27M</t>
+          <t>+$6.88M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$7.66M</t>
+          <t>+$8.40M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1052,12 +1052,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>+$10.06M</t>
+          <t>+$11.17M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$13.48M</t>
+          <t>+$14.98M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1114,12 +1114,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$14.56M</t>
+          <t>+$16.42M</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+$16.24M</t>
+          <t>+$18.32M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>+$2.93M</t>
+          <t>+$3.61M</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>+$4.67M</t>
+          <t>+$5.75M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1164,24 +1164,24 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>98.59</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>775</v>
+        <v>7760</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$4.54M</t>
+          <t>+$2.73M</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+$4.55M</t>
+          <t>+$3.09M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1193,72 +1193,101 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
+        <v>98.59</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>775</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>+$4.54M</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>+$4.55M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>103.4</v>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B24" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>+$565.11K</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>+$646.68K</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>+$645.83K</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>+$739.06K</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>108.4</v>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B25" s="5" t="n">
         <v>7775</v>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>+$6.11M</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>+$6.18M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>+$7.13M</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>+$7.21M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G24"/>
+  <autoFilter ref="A1:G25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2686,7 +2715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2798,12 +2827,12 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>+$1.67M</t>
+          <t>+$1.69M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+$27.76M</t>
+          <t>+$28.05M</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -2870,12 +2899,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$16.55M</t>
+          <t>+$17.71M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>+$23.68M</t>
+          <t>+$25.35M</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -2908,12 +2937,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>+$12.28M</t>
+          <t>+$12.41M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$19.23M</t>
+          <t>+$19.43M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -2928,38 +2957,42 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>-16.6</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>7720</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>-$6.89M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>+$19.05M</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>+$16.42M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>+$18.32M</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3040,24 +3073,24 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>-51.7</v>
+        <v>23.4</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>760</v>
+        <v>7690</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>-$11.14M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>+$10.85M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$18.01M</t>
+          <t>+$18.04M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -3067,7 +3100,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3078,24 +3111,24 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>48.5</v>
+        <v>-51.7</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>770</v>
+        <v>760</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>+$5.95M</t>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>-$11.14M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>+$17.42M</t>
+          <t>+$18.01M</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -3105,7 +3138,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3116,10 +3149,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-41.6</v>
+        <v>-16.6</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7625</v>
+        <v>7650</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
@@ -3128,12 +3161,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>-$10.85M</t>
+          <t>-$6.49M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$17.41M</t>
+          <t>+$17.94M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3150,74 +3183,70 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>23.4</v>
+        <v>48.5</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>7690</v>
+        <v>770</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>+$5.95M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>+$17.42M</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>-41.6</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>7625</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>+$10.25M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>+$17.04M</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>7720</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$14.56M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>+$16.24M</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>-$10.10M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>+$16.21M</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3226,36 +3255,32 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-36.6</v>
+        <v>43.4</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>7630</v>
+        <v>7710</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>-$11.25M</t>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$11.17M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+$15.80M</t>
+          <t>+$14.98M</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -3264,32 +3289,36 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>43.4</v>
+        <v>-36.6</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>7710</v>
+        <v>7630</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>+$10.06M</t>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>-$10.37M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+$13.48M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3492,12 +3521,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-$8.49M</t>
+          <t>-$7.98M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$10.25M</t>
+          <t>+$9.63M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -3550,40 +3579,40 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
-        <v>-51.6</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>7615</v>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="B24" s="2" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>7685</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>-$2.63M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>+$9.18M</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>+$684.63K</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>+$9.39M</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3628,74 +3657,74 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>-9.859999999999999</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>709</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$1.22M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$8.97M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>7685</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="B27" s="5" t="n">
+        <v>-51.6</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>7615</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$662.78K</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>+$9.09M</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>-9.859999999999999</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>709</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>-$1.22M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>+$8.97M</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-$2.46M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$8.60M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3704,28 +3733,28 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>2977.76</v>
+        <v>38.4</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>296</v>
+        <v>7705</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>-$5.01M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$6.88M</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+$8.36M</t>
+          <t>+$8.40M</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3746,10 +3775,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>2967.7</v>
+        <v>2977.76</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
@@ -3758,12 +3787,12 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>-$2.51M</t>
+          <t>-$5.01M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$7.74M</t>
+          <t>+$8.36M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -3773,7 +3802,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3784,10 +3813,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>38.4</v>
+        <v>28.4</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>7705</v>
+        <v>7695</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
@@ -3796,12 +3825,12 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>+$6.27M</t>
+          <t>+$3.95M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$7.66M</t>
+          <t>+$8.10M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -3818,28 +3847,28 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>28.4</v>
+        <v>2967.7</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>7695</v>
+        <v>295</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>+$3.67M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>-$2.51M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$7.52M</t>
+          <t>+$7.74M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -3849,7 +3878,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3872,12 +3901,12 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>+$6.11M</t>
+          <t>+$7.13M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$6.18M</t>
+          <t>+$7.21M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -3894,112 +3923,108 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-133.13</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>706</v>
+        <v>7750</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>-$491.18K</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>+$3.61M</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+$5.69M</t>
+          <t>+$5.75M</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>-133.13</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>706</v>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>-$491.18K</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>+$5.69M</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>2947.58</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="2" t="n">
         <v>293</v>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>+$2.32M</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>+$5.23M</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>442.14</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>720</v>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>+$4.38M</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>+$5.11M</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4012,70 +4037,74 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
+        <v>442.14</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>720</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>+$4.38M</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>+$5.11M</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
         <v>-379.68</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C37" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>-$4.08M</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>+$4.76M</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>+$2.93M</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>+$4.67M</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4146,78 +4175,74 @@
       <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>7760</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>+$2.73M</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>+$3.09M</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n">
+      <c r="B41" s="5" t="n">
         <v>-585.13</v>
       </c>
-      <c r="C40" s="5" t="n">
+      <c r="C41" s="5" t="n">
         <v>695</v>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>-$2.78M</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>+$2.88M</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>-297.5</v>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>702</v>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>-$632.27K</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>+$1.40M</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4228,24 +4253,24 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>401.05</v>
+        <v>-297.5</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>719</v>
+        <v>702</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>+$463.01K</t>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>-$632.27K</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>+$1.16M</t>
+          <t>+$1.40M</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -4255,7 +4280,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4266,24 +4291,24 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>-461.86</v>
+        <v>401.05</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>698</v>
+        <v>719</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>-$132.60K</t>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>+$463.01K</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>+$925.87K</t>
+          <t>+$1.16M</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -4293,83 +4318,83 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>-461.86</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>698</v>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>-$132.60K</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>+$925.87K</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B45" s="2" t="n">
         <v>103.4</v>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C45" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>+$565.11K</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$646.68K</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>+$645.83K</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>+$739.06K</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>-63.33</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>29080</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>+$342.73K</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>+$522.25K</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4380,24 +4405,24 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>6.67</v>
+        <v>-63.33</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>29150</v>
+        <v>29080</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>-$30.60K</t>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>+$342.73K</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>+$432.78K</t>
+          <t>+$522.25K</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -4407,7 +4432,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4418,10 +4443,10 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>-43.33</v>
+        <v>6.67</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>29100</v>
+        <v>29150</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4430,12 +4455,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>-$104.92K</t>
+          <t>-$30.60K</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>+$314.75K</t>
+          <t>+$432.78K</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -4456,10 +4481,10 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>56.67</v>
+        <v>-43.33</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>29200</v>
+        <v>29100</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4468,12 +4493,12 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>-$8.74K</t>
+          <t>-$104.92K</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>+$209.83K</t>
+          <t>+$314.75K</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -4494,70 +4519,70 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>-$8.74K</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>+$209.83K</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
         <v>106.67</v>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C50" s="5" t="n">
         <v>29250</v>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>+$73.44K</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>+$204.00K</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>-13.33</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>29130</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>+$174.86K</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4570,10 +4595,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>156.67</v>
+        <v>-13.33</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>29300</v>
+        <v>29130</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
@@ -4582,20 +4607,24 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>+$68.20K</t>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>+$166.70K</t>
+          <t>+$174.86K</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -4604,36 +4633,32 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>-18.33</v>
+        <v>156.67</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>29125</v>
+        <v>29300</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>-$91.80K</t>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>+$68.20K</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$153.00K</t>
+          <t>+$166.70K</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -4642,72 +4667,72 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
+        <v>-18.33</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>29125</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>-$91.80K</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$153.00K</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>146.67</v>
       </c>
-      <c r="C53" s="2" t="n">
+      <c r="C54" s="2" t="n">
         <v>29290</v>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>+$150.96K</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>+$150.96K</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n">
-        <v>-143.33</v>
-      </c>
-      <c r="C54" s="5" t="n">
-        <v>29000</v>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>-$102.29K</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>+$132.60K</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4718,24 +4743,24 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>36.67</v>
+        <v>-143.33</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>29180</v>
+        <v>29000</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>-$102.29K</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>+$131.14K</t>
+          <t>+$132.60K</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -4745,7 +4770,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4756,10 +4781,10 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>76.67</v>
+        <v>36.67</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>29220</v>
+        <v>29180</v>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
@@ -4768,12 +4793,12 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>+$65.57K</t>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>+$118.03K</t>
+          <t>+$131.14K</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -4794,70 +4819,74 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>29220</v>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>+$65.57K</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>+$118.03K</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
         <v>-193.33</v>
       </c>
-      <c r="C57" s="5" t="n">
+      <c r="C58" s="5" t="n">
         <v>28950</v>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E58" s="7" t="inlineStr">
         <is>
           <t>-$96.17K</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>+$102.58K</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>-93.33</v>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>29050</v>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>-$57.12K</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>+$89.76K</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -4866,10 +4895,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>26.67</v>
+        <v>-93.33</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>29170</v>
+        <v>29050</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
@@ -4878,12 +4907,12 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>-$26.23K</t>
+          <t>-$57.12K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$87.43K</t>
+          <t>+$89.76K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -4900,24 +4929,24 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>181.67</v>
+        <v>26.67</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>29325</v>
+        <v>29170</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>+$62.95K</t>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>-$26.23K</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$87.43K</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -4934,36 +4963,32 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>81.67</v>
+        <v>181.67</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>29225</v>
+        <v>29325</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-$61.20K</t>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$62.95K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$61.20K</t>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -4972,19 +4997,19 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>131.67</v>
+        <v>81.67</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>29275</v>
+        <v>29225</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>+$4.08K</t>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>-$61.20K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -5010,10 +5035,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>-33.33</v>
+        <v>131.67</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>29110</v>
+        <v>29275</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
@@ -5022,12 +5047,12 @@
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>+$26.23K</t>
+          <t>+$4.08K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$34.97K</t>
+          <t>+$61.20K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -5037,7 +5062,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5048,39 +5073,77 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
+        <v>-33.33</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>29110</v>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>+$26.23K</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>+$34.97K</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
         <v>-183.33</v>
       </c>
-      <c r="C64" s="2" t="n">
+      <c r="C65" s="2" t="n">
         <v>28960</v>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>-$6.41K</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>+$6.41K</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H64"/>
+  <autoFilter ref="A1:H65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
GEX delta update 2026-09-03 13:09
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-03.xlsx
+++ b/gex_pivot_levels_2026-09-03.xlsx
@@ -10,13 +10,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ES" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NQ" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTY" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Pivots'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -528,7 +532,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>-116.6</v>
+        <v>7565.4</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>7550</v>
@@ -557,7 +561,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>-66.59999999999999</v>
+        <v>7615.4</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>7600</v>
@@ -569,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$9.01M</t>
+          <t>-$9.27M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$10.87M</t>
+          <t>+$11.18M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -590,7 +594,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>-51.7</v>
+        <v>7630.3</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>760</v>
@@ -619,7 +623,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>-51.6</v>
+        <v>7630.4</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>7615</v>
@@ -652,7 +656,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>-41.6</v>
+        <v>7640.4</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>7625</v>
@@ -664,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$11.41M</t>
+          <t>-$11.59M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$18.31M</t>
+          <t>+$18.61M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -681,7 +685,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>-36.6</v>
+        <v>7645.4</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>7630</v>
@@ -693,12 +697,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$11.78M</t>
+          <t>-$11.95M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$16.55M</t>
+          <t>+$16.79M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -714,7 +718,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>-31.66</v>
+        <v>7650.34</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>762</v>
@@ -747,7 +751,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>-26.6</v>
+        <v>7655.4</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>7640</v>
@@ -780,7 +784,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>-16.6</v>
+        <v>7665.4</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>7650</v>
@@ -792,12 +796,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$7.29M</t>
+          <t>-$7.37M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$20.16M</t>
+          <t>+$20.38M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -813,7 +817,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>-11.62</v>
+        <v>7670.38</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>764</v>
@@ -846,7 +850,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>-1.6</v>
+        <v>7680.4</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>765</v>
@@ -879,7 +883,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>8.4</v>
+        <v>7690.4</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>7675</v>
@@ -908,7 +912,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>13.4</v>
+        <v>7695.4</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>7680</v>
@@ -941,7 +945,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>18.4</v>
+        <v>7700.4</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>7685</v>
@@ -953,12 +957,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$655.49K</t>
+          <t>+$648.21K</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$8.99M</t>
+          <t>+$8.89M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -974,7 +978,7 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>23.4</v>
+        <v>7705.4</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>7690</v>
@@ -1007,7 +1011,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>28.4</v>
+        <v>7710.4</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>7695</v>
@@ -1019,12 +1023,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$3.53M</t>
+          <t>+$3.48M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$7.23M</t>
+          <t>+$7.14M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1040,7 +1044,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>28.46</v>
+        <v>7710.46</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>768</v>
@@ -1073,7 +1077,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>33.4</v>
+        <v>7715.4</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>7700</v>
@@ -1106,7 +1110,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>38.4</v>
+        <v>7720.4</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>7705</v>
@@ -1118,12 +1122,12 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>+$5.87M</t>
+          <t>+$5.77M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$7.17M</t>
+          <t>+$7.04M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1139,7 +1143,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>38.48</v>
+        <v>7720.48</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>769</v>
@@ -1171,54 +1175,58 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>43.4</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>7710</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>+$9.31M</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>+$12.49M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
+      <c r="A22" s="5" t="n">
+        <v>7730.5</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>+$26.55M</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>+$39.84M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>48.5</v>
+        <v>7735.4</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>770</v>
+        <v>7720</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>+$26.55M</t>
+          <t>+$13.07M</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>+$39.84M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1233,135 +1241,73 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>7720</v>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="A24" s="2" t="n">
+        <v>7785.4</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>+$13.44M</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>+$14.99M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>+$565.11K</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>+$646.68K</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>7790.4</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7775</v>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>+$6.11M</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>+$6.18M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>+$2.93M</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>+$4.67M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>103.4</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>7770</v>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>+$565.11K</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>+$646.68K</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="n">
-        <v>108.4</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>7775</v>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>+$6.11M</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>+$6.18M</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G27"/>
+  <autoFilter ref="A1:G25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1424,7 +1370,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>-379.68</v>
+        <v>28852.32</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>700</v>
@@ -1457,7 +1403,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>-338.59</v>
+        <v>28893.41</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>701</v>
@@ -1490,7 +1436,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>-193.33</v>
+        <v>29038.67</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>28950</v>
@@ -1523,7 +1469,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>-183.33</v>
+        <v>29048.67</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>28960</v>
@@ -1556,7 +1502,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>-174.23</v>
+        <v>29057.77</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>705</v>
@@ -1589,7 +1535,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>-143.33</v>
+        <v>29088.67</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>29000</v>
@@ -1622,7 +1568,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>-93.33</v>
+        <v>29138.67</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>29050</v>
@@ -1651,7 +1597,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>-63.33</v>
+        <v>29168.67</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>29080</v>
@@ -1684,7 +1630,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>-43.33</v>
+        <v>29188.67</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>29100</v>
@@ -1717,7 +1663,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>-33.33</v>
+        <v>29198.67</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>29110</v>
@@ -1750,7 +1696,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>-18.33</v>
+        <v>29213.67</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>29125</v>
@@ -1783,7 +1729,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>-13.33</v>
+        <v>29218.67</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>29130</v>
@@ -1816,7 +1762,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>-9.859999999999999</v>
+        <v>29222.14</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>709</v>
@@ -1845,7 +1791,7 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>6.67</v>
+        <v>29238.67</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>29150</v>
@@ -1878,7 +1824,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>26.67</v>
+        <v>29258.67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>29170</v>
@@ -1907,7 +1853,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>36.67</v>
+        <v>29268.67</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>29180</v>
@@ -1940,7 +1886,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>56.67</v>
+        <v>29288.67</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>29200</v>
@@ -1973,7 +1919,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>76.67</v>
+        <v>29308.67</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>29220</v>
@@ -2006,7 +1952,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>81.67</v>
+        <v>29313.67</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>29225</v>
@@ -2039,7 +1985,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>106.67</v>
+        <v>29338.67</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>29250</v>
@@ -2072,7 +2018,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>113.41</v>
+        <v>29345.41</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>712</v>
@@ -2105,7 +2051,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>131.67</v>
+        <v>29363.67</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>29275</v>
@@ -2138,7 +2084,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>146.67</v>
+        <v>29378.67</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>29290</v>
@@ -2171,7 +2117,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>156.67</v>
+        <v>29388.67</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>29300</v>
@@ -2200,7 +2146,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>181.67</v>
+        <v>29413.67</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>29325</v>
@@ -2229,7 +2175,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>195.59</v>
+        <v>29427.59</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>714</v>
@@ -2262,7 +2208,7 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
-        <v>236.68</v>
+        <v>29468.68</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>715</v>
@@ -2295,7 +2241,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>442.14</v>
+        <v>29674.14</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>720</v>
@@ -2554,11 +2500,936 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="006C5CE7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Futures Strike</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ETF Strike</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Net GEX</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Abs GEX</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Pivot Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>+$117.19K</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>+$667.19K</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>+$2.86M</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>89.03</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>+$3.28M</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>+$3.84M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>90.31999999999999</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-$3.36M</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>+$7.81M</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>93.54000000000001</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>+$6.91M</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>+$6.96M</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>96.12</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>96.77</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>+$3.60M</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>+$3.62M</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="006C5CE7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Futures Strike</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ETF Strike</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Net GEX</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Abs GEX</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Pivot Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>4264.78</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>-$3.92M</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>+$4.03M</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>4310.64</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$588.78K</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>+$887.50K</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>4379.51</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-$664.83K</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>+$664.83K</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4401.74</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>396</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-$166.32K</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>+$849.56K</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>4402.35</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>-$8.30M</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>+$9.17M</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4412.85</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-$125.18K</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$261.10K</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4435.08</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>399</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>-$2.02M</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>+$2.73M</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>4479.55</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>403</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>-$344.97K</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>+$2.90M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>4490.66</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>404</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>+$386.89K</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$1.38M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4494.07</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-$1.61M</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>+$6.14M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4501.78</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>405</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>-$510.98K</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>+$3.81M</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>4524.01</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>407</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>+$864.86K</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>+$1.30M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>4535.12</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>408</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-$181.95K</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$1.12M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>4539.93</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>-$5.51M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$8.71M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>4557.35</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>+$420.39K</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>+$795.77K</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>4631.64</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>+$8.07M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$10.01M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>4677.5</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>+$8.44M</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>+$9.15M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FDCB6E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2620,7 +3491,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>-1.6</v>
+        <v>7680.4</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>765</v>
@@ -2658,7 +3529,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-11.62</v>
+        <v>7670.38</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>764</v>
@@ -2696,7 +3567,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>28.46</v>
+        <v>7710.46</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>768</v>
@@ -2734,7 +3605,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-9.859999999999999</v>
+        <v>29222.14</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>709</v>
@@ -2768,7 +3639,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>-31.66</v>
+        <v>7650.34</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>762</v>
@@ -2806,7 +3677,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>48.5</v>
+        <v>7730.5</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>770</v>
@@ -2844,7 +3715,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-51.7</v>
+        <v>7630.3</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>760</v>
@@ -2912,7 +3783,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>236.68</v>
+        <v>29468.68</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>715</v>
@@ -2950,7 +3821,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>8.4</v>
+        <v>7690.4</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>7675</v>
@@ -3022,7 +3893,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>38.48</v>
+        <v>7720.48</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>769</v>
@@ -3060,7 +3931,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>33.4</v>
+        <v>7715.4</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>7700</v>
@@ -3098,7 +3969,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>-16.6</v>
+        <v>7665.4</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>7650</v>
@@ -3110,12 +3981,12 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>-$7.29M</t>
+          <t>-$7.37M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>+$20.16M</t>
+          <t>+$20.38M</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -3136,7 +4007,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-174.23</v>
+        <v>29057.77</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>705</v>
@@ -3174,7 +4045,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>13.4</v>
+        <v>7695.4</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>7680</v>
@@ -3212,7 +4083,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>113.41</v>
+        <v>29345.41</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>712</v>
@@ -3250,7 +4121,7 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-41.6</v>
+        <v>7640.4</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>7625</v>
@@ -3262,12 +4133,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$11.41M</t>
+          <t>-$11.59M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$18.31M</t>
+          <t>+$18.61M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -3284,7 +4155,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-36.6</v>
+        <v>7645.4</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>7630</v>
@@ -3296,12 +4167,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>-$11.78M</t>
+          <t>-$11.95M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$16.55M</t>
+          <t>+$16.79M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3322,7 +4193,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>23.4</v>
+        <v>7705.4</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>7690</v>
@@ -3360,7 +4231,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-26.6</v>
+        <v>7655.4</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>7640</v>
@@ -3398,7 +4269,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>53.4</v>
+        <v>7735.4</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>7720</v>
@@ -3410,12 +4281,12 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>+$13.44M</t>
+          <t>+$13.07M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>+$14.99M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -3468,64 +4339,68 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>43.4</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>7710</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>+$9.31M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$12.49M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>28852.32</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>-$10.22M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>-379.68</v>
+        <v>2917.4</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>700</v>
+        <v>290</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>-$10.22M</t>
+          <t>-$10.48M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$11.36M</t>
+          <t>+$11.25M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -3542,28 +4417,28 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2917.4</v>
+        <v>7615.4</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>290</v>
+        <v>7600</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>-$10.48M</t>
+          <t>-$9.27M</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>+$11.25M</t>
+          <t>+$11.18M</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -3578,38 +4453,38 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>-66.59999999999999</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-$9.01M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$10.87M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>29427.59</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$7.28M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$10.27M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3618,40 +4493,36 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>195.59</v>
+        <v>4631.64</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>714</v>
+        <v>101</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>+$7.28M</t>
+          <t>+$8.07M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$10.27M</t>
+          <t>+$10.01M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -3660,7 +4531,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>-51.6</v>
+        <v>7630.4</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>7615</v>
@@ -3692,38 +4563,38 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>7685</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>+$655.49K</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>+$8.99M</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>4402.35</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>-$8.30M</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>+$9.17M</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3732,62 +4603,66 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>442.14</v>
+        <v>4677.5</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>720</v>
+        <v>102</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>+$7.95M</t>
+          <t>+$8.44M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$8.75M</t>
+          <t>+$9.15M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>2927.46</v>
+        <v>7700.4</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>291</v>
+        <v>7685</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>-$4.91M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>+$648.21K</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+$7.42M</t>
+          <t>+$8.89M</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -3797,81 +4672,77 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>28.4</v>
+        <v>29674.14</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>7695</v>
+        <v>720</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>+$3.53M</t>
+          <t>+$7.95M</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+$7.23M</t>
+          <t>+$8.75M</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>7705</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>+$5.87M</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>+$7.17M</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>4539.93</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>-$5.51M</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>+$8.71M</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3880,28 +4751,28 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>108.4</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>7775</v>
+        <v>140</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>+$6.11M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>-$3.36M</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>+$6.18M</t>
+          <t>+$7.81M</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -3911,43 +4782,47 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>2927.46</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7750</v>
+        <v>291</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>+$2.93M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>-$4.91M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$4.67M</t>
+          <t>+$7.42M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -3956,58 +4831,62 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>-116.6</v>
+        <v>7710.4</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>7550</v>
+        <v>7695</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-$3.85M</t>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>+$3.48M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$4.11M</t>
+          <t>+$7.14M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>-338.59</v>
+        <v>7720.4</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>701</v>
+        <v>7705</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$3.46M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>+$5.77M</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$3.80M</t>
+          <t>+$7.04M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4017,73 +4896,73 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>93.54000000000001</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>+$6.91M</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>+$6.96M</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>103.4</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>7770</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>+$565.11K</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>+$646.68K</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>-63.33</v>
+        <v>7790.4</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>29080</v>
+        <v>7775</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>+$342.73K</t>
+          <t>+$6.11M</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>+$522.25K</t>
+          <t>+$6.18M</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -4098,106 +4977,102 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>29150</v>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>-$30.60K</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>+$432.78K</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>4494.07</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>-$1.61M</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>+$6.14M</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>-43.33</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>29100</v>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>-$104.92K</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>+$314.75K</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>7565.4</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>7550</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$3.85M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$4.11M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>56.67</v>
+        <v>4264.78</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>29200</v>
+        <v>93</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>-$8.74K</t>
+          <t>-$3.92M</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>+$209.83K</t>
+          <t>+$4.03M</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -4214,28 +5089,28 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>106.67</v>
+        <v>89.03</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>29250</v>
+        <v>138</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>+$73.44K</t>
+          <t>+$3.28M</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>+$204.00K</t>
+          <t>+$3.84M</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -4250,40 +5125,40 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="n">
-        <v>-13.33</v>
-      </c>
-      <c r="C46" s="2" t="n">
-        <v>29130</v>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>+$174.86K</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>4501.78</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>405</v>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>-$510.98K</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>+$3.81M</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4294,172 +5169,168 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>156.67</v>
+        <v>28893.41</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>29300</v>
+        <v>701</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>+$68.20K</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>-$3.46M</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>+$166.70K</t>
+          <t>+$3.80M</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>-18.33</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>29125</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>-$91.80K</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$153.00K</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>96.77</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>+$3.60M</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$3.62M</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>146.67</v>
+        <v>4479.55</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>29290</v>
+        <v>403</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>+$150.96K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>-$344.97K</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>+$150.96K</t>
+          <t>+$2.90M</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n">
-        <v>-143.33</v>
-      </c>
-      <c r="C50" s="5" t="n">
-        <v>29000</v>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>-$102.29K</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>+$132.60K</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$2.86M</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>36.67</v>
+        <v>4435.08</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>29180</v>
+        <v>399</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>-$2.02M</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>+$131.14K</t>
+          <t>+$2.73M</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -4469,342 +5340,1200 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>4490.66</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>404</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>+$386.89K</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$1.38M</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n">
-        <v>76.67</v>
-      </c>
-      <c r="C52" s="5" t="n">
-        <v>29220</v>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>+$65.57K</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>+$118.03K</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4524.01</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>407</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>+$864.86K</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>+$1.30M</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>-193.33</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>28950</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$96.17K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$102.58K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n">
-        <v>-93.33</v>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>29050</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>-$57.12K</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>+$89.76K</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>26.67</v>
+        <v>4535.12</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>29170</v>
+        <v>408</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>-$26.23K</t>
+          <t>-$181.95K</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$87.43K</t>
+          <t>+$1.12M</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>181.67</v>
+        <v>4310.64</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>29325</v>
+        <v>94</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>+$62.95K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>-$588.78K</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$887.50K</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>81.67</v>
+        <v>4401.74</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>29225</v>
+        <v>396</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-$61.20K</t>
+          <t>-$166.32K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$61.20K</t>
+          <t>+$849.56K</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>131.67</v>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>29275</v>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>+$4.08K</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>+$61.20K</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>4557.35</v>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>+$420.39K</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>+$795.77K</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>-33.33</v>
+        <v>83.87</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>29110</v>
+        <v>130</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>+$26.23K</t>
+          <t>+$117.19K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$34.97K</t>
+          <t>+$667.19K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>4379.51</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>-$664.83K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$664.83K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>7785.4</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$565.11K</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>+$646.68K</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n">
-        <v>-183.33</v>
-      </c>
-      <c r="C60" s="2" t="n">
+      <c r="B62" s="5" t="n">
+        <v>29168.67</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>29080</v>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>+$342.73K</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>+$522.25K</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>29238.67</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>29150</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>-$30.60K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$432.78K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>29188.67</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>29100</v>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-$104.92K</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>+$314.75K</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>4412.85</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>-$125.18K</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>+$261.10K</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>29288.67</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>-$8.74K</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>+$209.83K</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>29338.67</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>29250</v>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>+$73.44K</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>+$204.00K</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>29218.67</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>29130</v>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>+$174.86K</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>29388.67</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>29300</v>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>+$68.20K</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>+$166.70K</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>29213.67</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>29125</v>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>-$91.80K</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>+$153.00K</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>29378.67</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>29290</v>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>+$150.96K</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>+$150.96K</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>29088.67</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>29000</v>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>-$102.29K</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>+$132.60K</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>29268.67</v>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>29180</v>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>+$131.14K</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>29308.67</v>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>29220</v>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>+$65.57K</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>+$118.03K</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>29038.67</v>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>28950</v>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>-$96.17K</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>+$102.58K</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>29138.67</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>29050</v>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>-$57.12K</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>+$89.76K</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>29258.67</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>29170</v>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>-$26.23K</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>+$87.43K</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>29413.67</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>29325</v>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>+$62.95K</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>29313.67</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>29225</v>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>-$61.20K</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>+$61.20K</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>29363.67</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>29275</v>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>+$4.08K</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>+$61.20K</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>96.12</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>29198.67</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>29110</v>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>+$26.23K</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>+$34.97K</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>29048.67</v>
+      </c>
+      <c r="C83" s="2" t="n">
         <v>28960</v>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E83" s="4" t="inlineStr">
         <is>
           <t>-$6.41K</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>+$6.41K</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G83" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H83" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:H83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports 2026-09-03 13:16
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-03.xlsx
+++ b/gex_pivot_levels_2026-09-03.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$9.27M</t>
+          <t>-$8.75M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$11.18M</t>
+          <t>+$10.56M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$2.80M</t>
+          <t>-$2.69M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$9.77M</t>
+          <t>+$9.38M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$11.59M</t>
+          <t>-$11.03M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$18.61M</t>
+          <t>+$17.71M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$11.95M</t>
+          <t>-$11.43M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$16.79M</t>
+          <t>+$16.05M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -763,12 +763,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$3.00M</t>
+          <t>-$2.92M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$15.77M</t>
+          <t>+$15.37M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$7.37M</t>
+          <t>-$7.21M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$20.38M</t>
+          <t>+$19.93M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$1.71M</t>
+          <t>+$1.74M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$28.33M</t>
+          <t>+$28.91M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -924,12 +924,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$12.28M</t>
+          <t>+$12.67M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$19.23M</t>
+          <t>+$19.84M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$648.21K</t>
+          <t>+$677.34K</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$8.89M</t>
+          <t>+$9.29M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>+$9.89M</t>
+          <t>+$10.37M</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>+$16.44M</t>
+          <t>+$17.24M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$3.48M</t>
+          <t>+$3.67M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$7.14M</t>
+          <t>+$7.52M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>+$15.38M</t>
+          <t>+$16.36M</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$22.01M</t>
+          <t>+$23.29M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>+$5.77M</t>
+          <t>+$6.17M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$7.04M</t>
+          <t>+$7.54M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1175,139 +1175,197 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>7730.5</v>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>770</v>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>+$26.55M</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>+$39.84M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n">
+        <v>7725.4</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>7710</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>+$9.90M</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>+$13.20M</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
+        <v>7730.5</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>+$26.55M</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>+$39.84M</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
         <v>7735.4</v>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B24" s="5" t="n">
         <v>7720</v>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>+$13.07M</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>+$14.57M</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>+$14.18M</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>+$15.82M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>7765.4</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>+$2.93M</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>+$4.67M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>7785.4</v>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B26" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>+$565.11K</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>+$646.68K</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
+    <row r="27">
+      <c r="A27" s="5" t="n">
         <v>7790.4</v>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B27" s="5" t="n">
         <v>7775</v>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>+$6.11M</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>+$6.18M</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3429,7 +3487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3833,12 +3891,12 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>+$1.71M</t>
+          <t>+$1.74M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$28.33M</t>
+          <t>+$28.91M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3943,12 +4001,12 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>+$15.38M</t>
+          <t>+$16.36M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>+$22.01M</t>
+          <t>+$23.29M</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -3963,76 +4021,76 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>29057.77</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>705</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>-$14.46M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$20.02M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B16" s="5" t="n">
         <v>7665.4</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C16" s="5" t="n">
         <v>7650</v>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>-$7.37M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+$20.38M</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-$7.21M</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>+$19.93M</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>29057.77</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>705</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>-$14.46M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>+$20.02M</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4057,12 +4115,12 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>+$12.28M</t>
+          <t>+$12.67M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$19.23M</t>
+          <t>+$19.84M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4133,12 +4191,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$11.59M</t>
+          <t>-$11.03M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$18.61M</t>
+          <t>+$17.71M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4149,152 +4207,152 @@
       <c r="H19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="5" t="n">
+        <v>7705.4</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>7690</v>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>+$10.37M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>+$17.24M</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
         <v>7645.4</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C21" s="2" t="n">
         <v>7630</v>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>-$11.95M</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>+$16.79M</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>-$11.43M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>+$16.05M</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>7705.4</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>7690</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="B22" s="5" t="n">
+        <v>7735.4</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>7720</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$9.89M</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>+$16.44M</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>+$14.18M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>+$15.82M</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>7655.4</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C23" s="2" t="n">
         <v>7640</v>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>-$3.00M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>+$15.77M</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$2.92M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>+$15.37M</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>7735.4</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>7720</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$13.07M</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>+$14.57M</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4339,68 +4397,64 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>28852.32</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>700</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-$10.22M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>+$11.36M</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7725.4</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7710</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$9.90M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$13.20M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2917.4</v>
+        <v>28852.32</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>290</v>
+        <v>700</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>-$10.48M</t>
+          <t>-$10.22M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$11.25M</t>
+          <t>+$11.36M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -4417,74 +4471,74 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2917.4</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>290</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-$10.48M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$11.25M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B28" s="5" t="n">
         <v>7615.4</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C28" s="5" t="n">
         <v>7600</v>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>-$9.27M</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>+$11.18M</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>-$8.75M</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>+$10.56M</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>29427.59</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>714</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>+$7.28M</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>+$10.27M</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4493,100 +4547,100 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>29427.59</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>+$7.28M</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>+$10.27M</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>4631.64</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>+$8.07M</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>+$10.01M</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>7630.4</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>7615</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-$2.80M</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>+$9.77M</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>4402.35</v>
+        <v>7630.4</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>96</v>
+        <v>7615</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>-$8.30M</t>
+          <t>-$2.69M</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>+$9.17M</t>
+          <t>+$9.38M</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -4596,81 +4650,81 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>7700.4</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>7685</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>+$677.34K</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>+$9.29M</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
-        <v>4677.5</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>102</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="B33" s="5" t="n">
+        <v>4402.35</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>+$8.44M</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>+$9.15M</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>7700.4</v>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>7685</v>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>+$648.21K</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>+$8.89M</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>-$8.30M</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>+$9.17M</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4679,148 +4733,148 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>4677.5</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>+$8.44M</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>+$9.15M</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>29674.14</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>+$7.95M</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>+$8.75M</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>4539.93</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>99</v>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>-$5.51M</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>+$8.71M</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>4539.93</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>-$5.51M</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>+$8.71M</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B37" s="5" t="n">
         <v>90.31999999999999</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C37" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>-$3.36M</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>+$7.81M</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>2927.46</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>291</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>-$4.91M</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>+$7.42M</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4831,10 +4885,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>7710.4</v>
+        <v>7720.4</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>7695</v>
+        <v>7705</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
@@ -4843,12 +4897,12 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>+$3.48M</t>
+          <t>+$6.17M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$7.14M</t>
+          <t>+$7.54M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -4869,10 +4923,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>7720.4</v>
+        <v>7710.4</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>7705</v>
+        <v>7695</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
@@ -4881,12 +4935,12 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>+$5.77M</t>
+          <t>+$3.67M</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$7.04M</t>
+          <t>+$7.52M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4901,38 +4955,38 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>93.54000000000001</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>145</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="inlineStr">
-        <is>
-          <t>+$6.91M</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>+$6.96M</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>2927.46</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>-$4.91M</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>+$7.42M</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4941,74 +4995,74 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>93.54000000000001</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>+$6.91M</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>+$6.96M</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B42" s="5" t="n">
         <v>7790.4</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C42" s="5" t="n">
         <v>7775</v>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>+$6.11M</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>+$6.18M</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>4494.07</v>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-$1.61M</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>+$6.14M</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5017,112 +5071,108 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>4494.07</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$1.61M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$6.14M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B44" s="2" t="n">
+        <v>7765.4</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>+$2.93M</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>+$4.67M</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
         <v>7565.4</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C45" s="2" t="n">
         <v>7550</v>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>-$3.85M</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>+$4.11M</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>4264.78</v>
-      </c>
-      <c r="C44" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>-$3.92M</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>+$4.03M</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>89.03</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>138</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>+$3.28M</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>+$3.84M</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -5131,24 +5181,24 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>4501.78</v>
+        <v>4264.78</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>405</v>
+        <v>93</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>-$510.98K</t>
+          <t>-$3.92M</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>+$3.81M</t>
+          <t>+$4.03M</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -5163,38 +5213,38 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>28893.41</v>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>701</v>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>-$3.46M</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>+$3.80M</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>89.03</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>+$3.28M</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>+$3.84M</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5203,28 +5253,28 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>96.77</v>
+        <v>4501.78</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>150</v>
+        <v>405</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>+$3.60M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>-$510.98K</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>+$3.62M</t>
+          <t>+$3.81M</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -5234,115 +5284,119 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>28893.41</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>701</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>-$3.46M</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>+$3.80M</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>96.77</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>+$3.60M</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>+$3.62M</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
+      <c r="B51" s="2" t="n">
         <v>4479.55</v>
       </c>
-      <c r="C49" s="2" t="n">
+      <c r="C51" s="2" t="n">
         <v>403</v>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>-$344.97K</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>+$2.90M</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>87.09</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>+$1.28M</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>+$2.86M</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n">
-        <v>4435.08</v>
-      </c>
-      <c r="C51" s="5" t="n">
-        <v>399</v>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>-$2.02M</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>+$2.73M</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -5351,108 +5405,104 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$2.86M</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>4435.08</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>399</v>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>-$2.02M</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>+$2.73M</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C54" s="2" t="n">
         <v>155</v>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>+$1.42M</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>+$1.42M</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="n">
-        <v>4490.66</v>
-      </c>
-      <c r="C53" s="2" t="n">
-        <v>404</v>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>+$386.89K</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>+$1.38M</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n">
-        <v>4524.01</v>
-      </c>
-      <c r="C54" s="5" t="n">
-        <v>407</v>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>+$864.86K</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>+$1.30M</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -5461,24 +5511,24 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>4535.12</v>
+        <v>4490.66</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>-$181.95K</t>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>+$386.89K</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$1.12M</t>
+          <t>+$1.38M</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -5488,43 +5538,43 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
-        <v>4310.64</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>-$588.78K</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>+$887.50K</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="B56" s="5" t="n">
+        <v>4524.01</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>407</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>+$864.86K</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>+$1.30M</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5537,10 +5587,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>4401.74</v>
+        <v>4535.12</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
@@ -5549,54 +5599,58 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-$166.32K</t>
+          <t>-$181.95K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$849.56K</t>
+          <t>+$1.12M</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
-        <v>4557.35</v>
-      </c>
-      <c r="C58" s="5" t="n">
-        <v>410</v>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>+$420.39K</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>+$795.77K</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="B58" s="2" t="n">
+        <v>4310.64</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>-$588.78K</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>+$887.50K</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5605,28 +5659,28 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>83.87</v>
+        <v>4401.74</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>130</v>
+        <v>396</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>+$117.19K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>-$166.32K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$667.19K</t>
+          <t>+$849.56K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -5637,152 +5691,148 @@
       <c r="H59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n">
-        <v>4379.51</v>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>394</v>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="B60" s="5" t="n">
+        <v>4557.35</v>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>-$664.83K</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>+$664.83K</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>+$420.39K</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>+$795.77K</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$117.19K</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>+$667.19K</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>4379.51</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>-$664.83K</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>+$664.83K</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B61" s="2" t="n">
+      <c r="B63" s="2" t="n">
         <v>7785.4</v>
       </c>
-      <c r="C61" s="2" t="n">
+      <c r="C63" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E61" s="8" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>+$565.11K</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>+$646.68K</t>
         </is>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="n">
-        <v>29168.67</v>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>29080</v>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E62" s="9" t="inlineStr">
-        <is>
-          <t>+$342.73K</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>+$522.25K</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="n">
-        <v>29238.67</v>
-      </c>
-      <c r="C63" s="5" t="n">
-        <v>29150</v>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>-$30.60K</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>+$432.78K</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -5795,24 +5845,24 @@
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>29188.67</v>
+        <v>29168.67</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>29100</v>
+        <v>29080</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>-$104.92K</t>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>+$342.73K</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>+$314.75K</t>
+          <t>+$522.25K</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -5822,45 +5872,45 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>29238.67</v>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>29150</v>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>-$30.60K</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>+$432.78K</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="n">
-        <v>4412.85</v>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v>397</v>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>-$125.18K</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>+$261.10K</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5871,146 +5921,150 @@
         </is>
       </c>
       <c r="B66" s="5" t="n">
+        <v>29188.67</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>29100</v>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>-$104.92K</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>+$314.75K</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>4412.85</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>-$125.18K</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>+$261.10K</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="n">
         <v>29288.67</v>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="C68" s="5" t="n">
         <v>29200</v>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E68" s="7" t="inlineStr">
         <is>
           <t>-$8.74K</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>+$209.83K</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B67" s="5" t="n">
+      <c r="B69" s="5" t="n">
         <v>29338.67</v>
       </c>
-      <c r="C67" s="5" t="n">
+      <c r="C69" s="5" t="n">
         <v>29250</v>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E67" s="9" t="inlineStr">
+      <c r="E69" s="9" t="inlineStr">
         <is>
           <t>+$73.44K</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>+$204.00K</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="n">
-        <v>29218.67</v>
-      </c>
-      <c r="C68" s="2" t="n">
-        <v>29130</v>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>+$174.86K</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n">
-        <v>29388.67</v>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>29300</v>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>+$68.20K</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>+$166.70K</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -6019,24 +6073,24 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>29213.67</v>
+        <v>29218.67</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>29125</v>
+        <v>29130</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>-$91.80K</t>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>+$153.00K</t>
+          <t>+$174.86K</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -6046,7 +6100,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6057,108 +6111,104 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
+        <v>29388.67</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>29300</v>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>+$68.20K</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>+$166.70K</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>29213.67</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>29125</v>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>-$91.80K</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>+$153.00K</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>29378.67</v>
       </c>
-      <c r="C71" s="2" t="n">
+      <c r="C73" s="2" t="n">
         <v>29290</v>
       </c>
-      <c r="D71" s="3" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
+      <c r="E73" s="8" t="inlineStr">
         <is>
           <t>+$150.96K</t>
         </is>
       </c>
-      <c r="F71" s="3" t="inlineStr">
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>+$150.96K</t>
         </is>
       </c>
-      <c r="G71" s="3" t="inlineStr">
+      <c r="G73" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="n">
-        <v>29088.67</v>
-      </c>
-      <c r="C72" s="5" t="n">
-        <v>29000</v>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>-$102.29K</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>+$132.60K</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="n">
-        <v>29268.67</v>
-      </c>
-      <c r="C73" s="5" t="n">
-        <v>29180</v>
-      </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>+$69.94K</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="inlineStr">
-        <is>
-          <t>+$131.14K</t>
-        </is>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
+      <c r="H73" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -6171,24 +6221,24 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>29308.67</v>
+        <v>29088.67</v>
       </c>
       <c r="C74" s="5" t="n">
-        <v>29220</v>
+        <v>29000</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E74" s="9" t="inlineStr">
-        <is>
-          <t>+$65.57K</t>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-$102.29K</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>+$118.03K</t>
+          <t>+$132.60K</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -6198,7 +6248,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6209,104 +6259,112 @@
         </is>
       </c>
       <c r="B75" s="5" t="n">
+        <v>29268.67</v>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>29180</v>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>+$131.14K</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>29308.67</v>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>29220</v>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>+$65.57K</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>+$118.03K</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="n">
         <v>29038.67</v>
       </c>
-      <c r="C75" s="5" t="n">
+      <c r="C77" s="5" t="n">
         <v>28950</v>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D77" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="E77" s="7" t="inlineStr">
         <is>
           <t>-$96.17K</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <t>+$102.58K</t>
         </is>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G77" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="n">
-        <v>29138.67</v>
-      </c>
-      <c r="C76" s="2" t="n">
-        <v>29050</v>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>-$57.12K</t>
-        </is>
-      </c>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>+$89.76K</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="n">
-        <v>29258.67</v>
-      </c>
-      <c r="C77" s="2" t="n">
-        <v>29170</v>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-$26.23K</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
-        <is>
-          <t>+$87.43K</t>
-        </is>
-      </c>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6315,24 +6373,24 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>29413.67</v>
+        <v>29138.67</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>29325</v>
+        <v>29050</v>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t>+$62.95K</t>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>-$57.12K</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$89.76K</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -6349,10 +6407,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>29313.67</v>
+        <v>29258.67</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>29225</v>
+        <v>29170</v>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
@@ -6361,24 +6419,20 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>-$61.20K</t>
+          <t>-$26.23K</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>+$61.20K</t>
+          <t>+$87.43K</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -6387,10 +6441,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>29363.67</v>
+        <v>29413.67</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>29275</v>
+        <v>29325</v>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
@@ -6399,50 +6453,46 @@
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>+$4.08K</t>
+          <t>+$62.95K</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>+$61.20K</t>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>96.12</v>
+        <v>29313.67</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>149</v>
+        <v>29225</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t>+$48.82K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>-$61.20K</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>+$48.82K</t>
+          <t>+$61.20K</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -6463,10 +6513,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>29198.67</v>
+        <v>29363.67</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>29110</v>
+        <v>29275</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
@@ -6475,12 +6525,12 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>+$26.23K</t>
+          <t>+$4.08K</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>+$34.97K</t>
+          <t>+$61.20K</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -6490,50 +6540,126 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>96.12</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>+$48.82K</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B83" s="2" t="n">
+      <c r="B84" s="2" t="n">
+        <v>29198.67</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>29110</v>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>+$26.23K</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>+$34.97K</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
         <v>29048.67</v>
       </c>
-      <c r="C83" s="2" t="n">
+      <c r="C85" s="2" t="n">
         <v>28960</v>
       </c>
-      <c r="D83" s="3" t="inlineStr">
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
+      <c r="E85" s="4" t="inlineStr">
         <is>
           <t>-$6.41K</t>
         </is>
       </c>
-      <c r="F83" s="3" t="inlineStr">
+      <c r="F85" s="3" t="inlineStr">
         <is>
           <t>+$6.41K</t>
         </is>
       </c>
-      <c r="G83" s="3" t="inlineStr">
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H83" s="3" t="inlineStr">
+      <c r="H85" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H83"/>
+  <autoFilter ref="A1:H85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports 2026-09-03 13:47
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-03.xlsx
+++ b/gex_pivot_levels_2026-09-03.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$3.85M</t>
+          <t>-$3.08M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$4.11M</t>
+          <t>+$3.29M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$8.75M</t>
+          <t>-$7.46M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$10.56M</t>
+          <t>+$9.01M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$2.69M</t>
+          <t>-$2.35M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$9.38M</t>
+          <t>+$8.20M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$11.03M</t>
+          <t>-$9.91M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$17.71M</t>
+          <t>+$15.91M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$11.43M</t>
+          <t>-$10.37M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$16.05M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -751,10 +751,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>7655.4</v>
+        <v>7665.4</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>7640</v>
+        <v>7650</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -763,130 +763,122 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$2.92M</t>
+          <t>-$6.89M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$15.37M</t>
+          <t>+$19.05M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>7670.38</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>764</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$11.72M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$58.49M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>7665.4</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7680.4</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>765</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-$31.42M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$88.68M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>7690.4</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$7.21M</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>+$19.93M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>7670.38</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>764</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>-$11.72M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$58.49M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>7680.4</v>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>765</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>-$31.42M</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>+$88.68M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>+$1.83M</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$30.34M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>7690.4</v>
+        <v>7695.4</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7675</v>
+        <v>7680</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -895,27 +887,31 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$1.74M</t>
+          <t>+$13.57M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$28.91M</t>
+          <t>+$21.25M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>7695.4</v>
+        <v>7700.4</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7680</v>
+        <v>7685</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -924,12 +920,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$12.67M</t>
+          <t>+$742.89K</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$19.84M</t>
+          <t>+$10.19M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -939,195 +935,195 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7705.4</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7690</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>+$11.58M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$19.25M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>7700.4</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>7685</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>7710.4</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>7695</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>+$677.34K</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$9.29M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>+$4.19M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$8.58M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>7705.4</v>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>7690</v>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>+$10.37M</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>+$17.24M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>7710.4</v>
+        <v>7710.46</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7695</v>
+        <v>768</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>+$33.36M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$48.12M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>7715.4</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>+$3.67M</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>+$7.52M</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>+$18.65M</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>+$26.68M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>7720.4</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>7705</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>+$7.08M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$8.65M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>7710.46</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>768</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>+$33.36M</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$48.12M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>7715.4</v>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>7700</v>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>+$16.36M</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>+$23.29M</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>7720.4</v>
+        <v>7720.48</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7705</v>
+        <v>769</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>+$6.17M</t>
+          <t>+$5.25M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$7.54M</t>
+          <t>+$23.83M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1143,86 +1139,86 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>7720.48</v>
+        <v>7725.4</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>769</v>
+        <v>7710</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>+$15.23M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>7730.5</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>+$5.25M</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$23.83M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>7725.4</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>7710</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>+$9.90M</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>+$13.20M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>+$26.55M</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>+$39.84M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>7730.5</v>
+        <v>7735.4</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>770</v>
+        <v>7720</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>+$26.55M</t>
+          <t>+$16.05M</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>+$39.84M</t>
+          <t>+$17.90M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1237,44 +1233,40 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
-        <v>7735.4</v>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>7720</v>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="A24" s="2" t="n">
+        <v>7765.4</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>+$14.18M</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>+$15.82M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>+$3.16M</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>+$5.03M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>7765.4</v>
+        <v>7785.4</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>7750</v>
+        <v>7770</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -1283,27 +1275,31 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>+$2.93M</t>
+          <t>+$645.83K</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>+$4.67M</t>
+          <t>+$739.06K</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>7785.4</v>
+        <v>7790.4</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7770</v>
+        <v>7775</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
@@ -1312,60 +1308,23 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>+$565.11K</t>
+          <t>+$6.11M</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>+$646.68K</t>
+          <t>+$6.18M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="n">
-        <v>7790.4</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>7775</v>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>+$6.11M</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>+$6.18M</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G27"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3487,7 +3446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3891,12 +3850,12 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>+$1.74M</t>
+          <t>+$1.83M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$28.91M</t>
+          <t>+$30.34M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3945,190 +3904,190 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="5" t="n">
+        <v>7715.4</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>+$18.65M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>+$26.68M</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
         <v>7720.48</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C14" s="2" t="n">
         <v>769</v>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>+$5.25M</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>+$23.83M</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>7715.4</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$16.36M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>+$23.29M</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>7695.4</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>7680</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$13.57M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$21.25M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B16" s="2" t="n">
         <v>29057.77</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C16" s="2" t="n">
         <v>705</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>-$14.46M</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>+$20.02M</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>7665.4</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="B17" s="5" t="n">
+        <v>7705.4</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>7690</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-$7.21M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$19.93M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>+$11.58M</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>+$19.25M</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>7695.4</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>7680</v>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>+$12.67M</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>+$19.84M</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4179,10 +4138,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7640.4</v>
+        <v>7665.4</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>7625</v>
+        <v>7650</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
@@ -4191,12 +4150,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$11.03M</t>
+          <t>-$6.89M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$17.71M</t>
+          <t>+$19.05M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4213,10 +4172,10 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>7705.4</v>
+        <v>7735.4</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>7690</v>
+        <v>7720</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -4225,12 +4184,12 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>+$10.37M</t>
+          <t>+$16.05M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$17.24M</t>
+          <t>+$17.90M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -4251,10 +4210,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>7645.4</v>
+        <v>7640.4</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>7630</v>
+        <v>7625</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
@@ -4263,62 +4222,54 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>-$11.43M</t>
+          <t>-$9.91M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>+$16.05M</t>
+          <t>+$15.91M</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
-        <v>7735.4</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>7720</v>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="B22" s="2" t="n">
+        <v>7725.4</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>7710</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>+$14.18M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>+$15.82M</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>+$15.23M</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -4327,10 +4278,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>7655.4</v>
+        <v>7645.4</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>7640</v>
+        <v>7630</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
@@ -4339,12 +4290,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>-$2.92M</t>
+          <t>-$10.37M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+$15.37M</t>
+          <t>+$14.57M</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -4354,7 +4305,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4397,148 +4348,152 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7725.4</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>7710</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>+$9.90M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$13.20M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>28852.32</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>-$10.22M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2917.4</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>290</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-$10.48M</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>+$11.25M</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>28852.32</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>700</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="B27" s="2" t="n">
+        <v>29427.59</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>-$10.22M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$11.36M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>+$7.28M</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>+$10.27M</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>2917.4</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>290</v>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>-$10.48M</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>+$11.25M</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>7615.4</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>7700.4</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7685</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-$8.75M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$10.56M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$742.89K</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$10.19M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4547,294 +4502,294 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>4631.64</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>+$8.07M</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>+$10.01M</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>4402.35</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-$8.30M</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>+$9.17M</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>4677.5</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>+$8.44M</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>+$9.15M</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7615.4</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>-$7.46M</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>+$9.01M</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
-        <v>29427.59</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>714</v>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="B33" s="2" t="n">
+        <v>29674.14</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>+$7.28M</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>+$10.27M</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>+$7.95M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$8.75M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>4539.93</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>-$5.51M</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>+$8.71M</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>4631.64</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>101</v>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>+$8.07M</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>+$10.01M</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>7630.4</v>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>7615</v>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>-$2.69M</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>+$9.38M</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>7700.4</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>7685</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>+$677.34K</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>+$9.29M</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>4402.35</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>96</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>-$8.30M</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>+$9.17M</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>4677.5</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>102</v>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>+$8.44M</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>+$9.15M</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>29674.14</v>
+        <v>7720.4</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>720</v>
+        <v>7705</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>+$7.95M</t>
+          <t>+$7.08M</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>+$8.75M</t>
+          <t>+$8.65M</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>4539.93</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>99</v>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>-$5.51M</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>+$8.71M</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>7710.4</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>7695</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>+$4.19M</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>+$8.58M</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4843,74 +4798,74 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>7630.4</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>7615</v>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>-$2.35M</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>+$8.20M</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B38" s="5" t="n">
         <v>90.31999999999999</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C38" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>-$3.36M</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>+$7.81M</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>7720.4</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>7705</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>+$6.17M</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>+$7.54M</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4919,150 +4874,146 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>2927.46</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>-$4.91M</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>+$7.42M</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>93.54000000000001</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>+$6.91M</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>+$6.96M</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>7710.4</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>7695</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="B41" s="2" t="n">
+        <v>7790.4</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>7775</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>+$3.67M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$7.52M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>+$6.11M</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>+$6.18M</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>4494.07</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>-$1.61M</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>+$6.14M</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>2927.46</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>291</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>-$4.91M</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>+$7.42M</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>93.54000000000001</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>145</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>+$6.91M</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>+$6.96M</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>7790.4</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>7775</v>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E42" s="9" t="inlineStr">
-        <is>
-          <t>+$6.11M</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>+$6.18M</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5071,108 +5022,112 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>7765.4</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>+$3.16M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$5.03M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
-        <v>4494.07</v>
-      </c>
-      <c r="C43" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="B44" s="5" t="n">
+        <v>4264.78</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>-$1.61M</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>+$6.14M</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>-$3.92M</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>+$4.03M</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>89.03</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>+$3.28M</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>+$3.84M</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>7765.4</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>+$2.93M</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$4.67M</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>7565.4</v>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>7550</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>-$3.85M</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>+$4.11M</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -5181,24 +5136,24 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>4264.78</v>
+        <v>4501.78</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>93</v>
+        <v>405</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>-$3.92M</t>
+          <t>-$510.98K</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>+$4.03M</t>
+          <t>+$3.81M</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -5213,38 +5168,38 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="n">
-        <v>89.03</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>138</v>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>+$3.28M</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>+$3.84M</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>28893.41</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>701</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>-$3.46M</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>+$3.80M</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5253,28 +5208,28 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>4501.78</v>
+        <v>96.77</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>405</v>
+        <v>150</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>-$510.98K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>+$3.60M</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>+$3.81M</t>
+          <t>+$3.62M</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -5284,299 +5239,295 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>28893.41</v>
+        <v>7565.4</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>701</v>
+        <v>7550</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>-$3.46M</t>
+          <t>-$3.08M</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>+$3.80M</t>
+          <t>+$3.29M</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n">
-        <v>96.77</v>
-      </c>
-      <c r="C50" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>+$3.60M</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>+$3.62M</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>4479.55</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>403</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>-$344.97K</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$2.90M</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>+$2.86M</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n">
-        <v>4479.55</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>403</v>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="B52" s="5" t="n">
+        <v>4435.08</v>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>399</v>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>-$344.97K</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>+$2.90M</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>-$2.02M</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>+$2.73M</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$1.42M</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>87.09</v>
-      </c>
-      <c r="C52" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>+$1.28M</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>+$2.86M</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>4435.08</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>399</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$2.02M</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$2.73M</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>100</v>
+        <v>4490.66</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>155</v>
+        <v>404</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>+$1.42M</t>
+          <t>+$386.89K</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$1.42M</t>
+          <t>+$1.38M</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B55" s="2" t="n">
-        <v>4490.66</v>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>404</v>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="B55" s="5" t="n">
+        <v>4524.01</v>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>407</v>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>+$386.89K</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>+$1.38M</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>+$864.86K</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>+$1.30M</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>4535.12</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>408</v>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>-$181.95K</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>+$1.12M</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="n">
-        <v>4524.01</v>
-      </c>
-      <c r="C56" s="5" t="n">
-        <v>407</v>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>+$864.86K</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>+$1.30M</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5587,24 +5538,24 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>4535.12</v>
+        <v>4310.64</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>408</v>
+        <v>94</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-$181.95K</t>
+          <t>-$588.78K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$1.12M</t>
+          <t>+$887.50K</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -5614,7 +5565,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5625,106 +5576,106 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>4310.64</v>
+        <v>4401.74</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>94</v>
+        <v>396</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>-$588.78K</t>
+          <t>-$166.32K</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$887.50K</t>
+          <t>+$849.56K</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>4557.35</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>+$420.39K</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>+$795.77K</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>7785.4</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>+$645.83K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$739.06K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n">
-        <v>4401.74</v>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>396</v>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>-$166.32K</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>+$849.56K</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>4557.35</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>410</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>+$420.39K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$795.77K</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5801,40 +5752,40 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>7785.4</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>7770</v>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>+$565.11K</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>+$646.68K</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>29168.67</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>29080</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>+$342.73K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$522.25K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5845,24 +5796,24 @@
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>29168.67</v>
+        <v>29238.67</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>29080</v>
+        <v>29150</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>+$342.73K</t>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-$30.60K</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>+$522.25K</t>
+          <t>+$432.78K</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -5872,7 +5823,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5883,10 +5834,10 @@
         </is>
       </c>
       <c r="B65" s="5" t="n">
-        <v>29238.67</v>
+        <v>29188.67</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>29150</v>
+        <v>29100</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
@@ -5895,12 +5846,12 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>-$30.60K</t>
+          <t>-$104.92K</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>+$432.78K</t>
+          <t>+$314.75K</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -5915,78 +5866,78 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>4412.85</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>-$125.18K</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>+$261.10K</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n">
-        <v>29188.67</v>
-      </c>
-      <c r="C66" s="5" t="n">
-        <v>29100</v>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="B67" s="5" t="n">
+        <v>29288.67</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
-        <is>
-          <t>-$104.92K</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>+$314.75K</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>-$8.74K</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>+$209.83K</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="n">
-        <v>4412.85</v>
-      </c>
-      <c r="C67" s="2" t="n">
-        <v>397</v>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-$125.18K</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>+$261.10K</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5997,24 +5948,24 @@
         </is>
       </c>
       <c r="B68" s="5" t="n">
-        <v>29288.67</v>
+        <v>29338.67</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>29200</v>
+        <v>29250</v>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr">
-        <is>
-          <t>-$8.74K</t>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>+$73.44K</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>+$209.83K</t>
+          <t>+$204.00K</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -6024,43 +5975,43 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B69" s="5" t="n">
-        <v>29338.67</v>
-      </c>
-      <c r="C69" s="5" t="n">
-        <v>29250</v>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="B69" s="2" t="n">
+        <v>29218.67</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>29130</v>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>+$73.44K</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>+$204.00K</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>+$174.86K</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -6073,10 +6024,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>29218.67</v>
+        <v>29388.67</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>29130</v>
+        <v>29300</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
@@ -6085,24 +6036,20 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$68.20K</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>+$174.86K</t>
+          <t>+$166.70K</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -6111,32 +6058,36 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>29388.67</v>
+        <v>29213.67</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>29300</v>
+        <v>29125</v>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>+$68.20K</t>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>-$91.80K</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>+$166.70K</t>
+          <t>+$153.00K</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -6145,24 +6096,24 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>29213.67</v>
+        <v>29378.67</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>29125</v>
+        <v>29290</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>-$91.80K</t>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>+$150.96K</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>+$153.00K</t>
+          <t>+$150.96K</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -6172,45 +6123,45 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>29088.67</v>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>29000</v>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>-$102.29K</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>+$132.60K</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="n">
-        <v>29378.67</v>
-      </c>
-      <c r="C73" s="2" t="n">
-        <v>29290</v>
-      </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>+$150.96K</t>
-        </is>
-      </c>
-      <c r="F73" s="3" t="inlineStr">
-        <is>
-          <t>+$150.96K</t>
-        </is>
-      </c>
-      <c r="G73" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H73" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6221,24 +6172,24 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>29088.67</v>
+        <v>29268.67</v>
       </c>
       <c r="C74" s="5" t="n">
-        <v>29000</v>
+        <v>29180</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E74" s="7" t="inlineStr">
-        <is>
-          <t>-$102.29K</t>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>+$132.60K</t>
+          <t>+$131.14K</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -6248,7 +6199,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6259,10 +6210,10 @@
         </is>
       </c>
       <c r="B75" s="5" t="n">
-        <v>29268.67</v>
+        <v>29308.67</v>
       </c>
       <c r="C75" s="5" t="n">
-        <v>29180</v>
+        <v>29220</v>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
@@ -6271,12 +6222,12 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$65.57K</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>+$131.14K</t>
+          <t>+$118.03K</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -6297,24 +6248,24 @@
         </is>
       </c>
       <c r="B76" s="5" t="n">
-        <v>29308.67</v>
+        <v>29038.67</v>
       </c>
       <c r="C76" s="5" t="n">
-        <v>29220</v>
+        <v>28950</v>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E76" s="9" t="inlineStr">
-        <is>
-          <t>+$65.57K</t>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-$96.17K</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>+$118.03K</t>
+          <t>+$102.58K</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -6324,47 +6275,43 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B77" s="5" t="n">
-        <v>29038.67</v>
-      </c>
-      <c r="C77" s="5" t="n">
-        <v>28950</v>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
+      <c r="B77" s="2" t="n">
+        <v>29138.67</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>29050</v>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E77" s="7" t="inlineStr">
-        <is>
-          <t>-$96.17K</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="inlineStr">
-        <is>
-          <t>+$102.58K</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>-$57.12K</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>+$89.76K</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6373,10 +6320,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>29138.67</v>
+        <v>29258.67</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>29050</v>
+        <v>29170</v>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
@@ -6385,12 +6332,12 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>-$57.12K</t>
+          <t>-$26.23K</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>+$89.76K</t>
+          <t>+$87.43K</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -6407,24 +6354,24 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>29258.67</v>
+        <v>29413.67</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>29170</v>
+        <v>29325</v>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-$26.23K</t>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>+$62.95K</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>+$87.43K</t>
+          <t>+$69.94K</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -6441,32 +6388,36 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>29413.67</v>
+        <v>29313.67</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>29325</v>
+        <v>29225</v>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>+$62.95K</t>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>-$61.20K</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>+$69.94K</t>
+          <t>+$61.20K</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -6475,19 +6426,19 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>29313.67</v>
+        <v>29363.67</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>29225</v>
+        <v>29275</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>-$61.20K</t>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>+$4.08K</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -6509,28 +6460,28 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>29363.67</v>
+        <v>96.12</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>29275</v>
+        <v>149</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>+$4.08K</t>
+          <t>+$48.82K</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>+$61.20K</t>
+          <t>+$48.82K</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -6547,28 +6498,28 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>96.12</v>
+        <v>29198.67</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>149</v>
+        <v>29110</v>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>+$48.82K</t>
+          <t>+$26.23K</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>+$48.82K</t>
+          <t>+$34.97K</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -6578,7 +6529,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6589,24 +6540,24 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>29198.67</v>
+        <v>29048.67</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>29110</v>
+        <v>28960</v>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>+$26.23K</t>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>-$6.41K</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>+$34.97K</t>
+          <t>+$6.41K</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -6620,46 +6571,8 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="n">
-        <v>29048.67</v>
-      </c>
-      <c r="C85" s="2" t="n">
-        <v>28960</v>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>-$6.41K</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>+$6.41K</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H85"/>
+  <autoFilter ref="A1:H84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>